<commit_message>
Update Excel chart template
</commit_message>
<xml_diff>
--- a/Reading-excel-chart-template.xlsx
+++ b/Reading-excel-chart-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eloise.Bartrop\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148E32B2-F363-4C2D-8CDA-6062A7EC7C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DCD378-05DA-45C5-A4AD-2C198102A28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{AF9D2CEB-64FD-4952-A634-7532AA11C33F}"/>
   </bookViews>
@@ -42,8 +42,100 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bartrop-Braybon, Eloise</author>
+  </authors>
+  <commentList>
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{C0325F13-9392-4F08-AACE-2AB987C89C90}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bartrop-Braybon, Eloise:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Bartrop-Braybon, Eloise</author>
+  </authors>
+  <commentList>
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{6C970E99-87EE-4FE2-88E0-256310B5A21F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bartrop-Braybon, Eloise:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F24" authorId="0" shapeId="0" xr:uid="{E355D821-BF7F-4C12-852D-C1E670D50C36}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bartrop-Braybon, Eloise:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="10">
   <si>
     <t>Customer name/description</t>
   </si>
@@ -79,7 +171,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,16 +214,45 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
+      <name val="3ds"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="20"/>
+      <b/>
+      <sz val="16"/>
       <color rgb="FFFF0000"/>
-      <name val="3ds"/>
+      <name val="Corbel"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="4" tint="-0.249977111117893"/>
+      <name val="Corbel"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -166,7 +287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -230,17 +351,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -475,71 +585,79 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,365 +922,365 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="38">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="39">
         <v>46098</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="38"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="38"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21">
+      <c r="A4" s="35">
         <v>100</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="17">
         <f>SUM(B4:E4)/4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="18">
         <f>-F4+H4</f>
         <v>100</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="31">
         <v>100</v>
       </c>
-      <c r="I4" s="38"/>
+      <c r="I4" s="39"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17">
+      <c r="A5" s="36">
         <v>95</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15">
+      <c r="B5" s="20"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="17">
         <f t="shared" ref="F5:F17" si="0">SUM(B5:E5)/4</f>
         <v>0</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="18">
         <f t="shared" ref="G5:G17" si="1">-F5+H5</f>
         <v>99</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="31">
         <v>99</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="39"/>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
+      <c r="A6" s="36">
         <v>90</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="13">
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="18">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="32">
         <v>97</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="39"/>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17">
+      <c r="A7" s="36">
         <v>80</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="32">
         <v>93</v>
       </c>
-      <c r="I7" s="38"/>
-      <c r="K7" s="22"/>
+      <c r="I7" s="39"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17">
+      <c r="A8" s="36">
         <v>70</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="32">
         <v>88</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="39"/>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
+      <c r="A9" s="36">
         <v>60</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="B9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="32">
         <v>81</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="36">
         <v>50</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="B10" s="21"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="32">
         <v>72</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17">
+      <c r="A11" s="36">
         <v>40</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
+      <c r="B11" s="21"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="32">
         <v>62</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="39"/>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
+      <c r="A12" s="36">
         <v>30</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="32">
         <v>51</v>
       </c>
-      <c r="I12" s="38"/>
+      <c r="I12" s="39"/>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17">
+      <c r="A13" s="36">
         <v>20</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="32">
         <v>37</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="39"/>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+      <c r="A14" s="36">
         <v>10</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="13">
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="32">
         <v>22</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+      <c r="A15" s="36">
         <v>5</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="H15" s="26">
+      <c r="H15" s="33">
         <v>13</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="36">
         <v>3</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="32">
         <v>9</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4">
+      <c r="A17" s="37">
         <v>1</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="10">
+      <c r="B17" s="24"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="27">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="34">
         <v>3</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="39">
+      <c r="A18" s="16">
         <v>123</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="32" t="s">
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="38" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1191,723 +1309,727 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="38">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="39">
         <v>46098</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="38"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="38"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21">
+      <c r="A4" s="35">
         <v>100</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="17">
         <f>SUM(B4:E4)/4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="18">
         <f>-F4+H4</f>
         <v>100</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="31">
         <v>100</v>
       </c>
-      <c r="I4" s="38"/>
+      <c r="I4" s="39"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17">
+      <c r="A5" s="36">
         <v>95</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15">
+      <c r="B5" s="20"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="17">
         <f t="shared" ref="F5:F17" si="0">SUM(B5:E5)/4</f>
         <v>0</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="18">
         <f t="shared" ref="G5:G17" si="1">-F5+H5</f>
         <v>99</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="31">
         <v>99</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="39"/>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
+      <c r="A6" s="36">
         <v>90</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="13">
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="18">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="32">
         <v>97</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="39"/>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17">
+      <c r="A7" s="36">
         <v>80</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="32">
         <v>93</v>
       </c>
-      <c r="I7" s="38"/>
-      <c r="K7" s="22"/>
+      <c r="I7" s="39"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17">
+      <c r="A8" s="36">
         <v>70</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="32">
         <v>88</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="39"/>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
+      <c r="A9" s="36">
         <v>60</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="B9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="32">
         <v>81</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="36">
         <v>50</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="B10" s="21"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="32">
         <v>72</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17">
+      <c r="A11" s="36">
         <v>40</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
+      <c r="B11" s="21"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="32">
         <v>62</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="39"/>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
+      <c r="A12" s="36">
         <v>30</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="32">
         <v>51</v>
       </c>
-      <c r="I12" s="38"/>
+      <c r="I12" s="39"/>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17">
+      <c r="A13" s="36">
         <v>20</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="32">
         <v>37</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="39"/>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+      <c r="A14" s="36">
         <v>10</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="13">
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="32">
         <v>22</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+      <c r="A15" s="36">
         <v>5</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="H15" s="26">
+      <c r="H15" s="33">
         <v>13</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="36">
         <v>3</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="32">
         <v>9</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4">
+      <c r="A17" s="37">
         <v>1</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="10">
+      <c r="B17" s="24"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="27">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="34">
         <v>3</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="39">
+      <c r="A18" s="16">
         <v>123</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="32" t="s">
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="38" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="38"/>
+      <c r="A19" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="39">
+        <v>46098</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="28" t="s">
+      <c r="A20" s="2"/>
+      <c r="B20" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="D20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E20" s="30" t="s">
+      <c r="E20" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="14" t="s">
+      <c r="G20" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="39"/>
     </row>
     <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="38"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="21">
+      <c r="A22" s="35">
         <v>100</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="15">
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="17">
         <f>SUM(B22:E22)/4</f>
         <v>0</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="18">
         <f>-F22+H22</f>
         <v>100</v>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="31">
         <v>100</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
+      <c r="A23" s="36">
         <v>95</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="15">
+      <c r="B23" s="20"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="17">
         <f t="shared" ref="F23:F35" si="2">SUM(B23:E23)/4</f>
         <v>0</v>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="18">
         <f t="shared" ref="G23:G35" si="3">-F23+H23</f>
         <v>99</v>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="31">
         <v>99</v>
       </c>
-      <c r="I23" s="38"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17">
+      <c r="A24" s="36">
         <v>90</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="15">
+      <c r="B24" s="21"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="18">
         <f t="shared" si="3"/>
         <v>97</v>
       </c>
-      <c r="H24" s="25">
+      <c r="H24" s="32">
         <v>97</v>
       </c>
-      <c r="I24" s="38"/>
+      <c r="I24" s="39"/>
     </row>
     <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="17">
+      <c r="A25" s="36">
         <v>80</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="15">
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="18">
         <f t="shared" si="3"/>
         <v>93</v>
       </c>
-      <c r="H25" s="25">
+      <c r="H25" s="32">
         <v>93</v>
       </c>
-      <c r="I25" s="38"/>
+      <c r="I25" s="39"/>
     </row>
     <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
+      <c r="A26" s="36">
         <v>70</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="15">
+      <c r="B26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="18">
         <f t="shared" si="3"/>
         <v>88</v>
       </c>
-      <c r="H26" s="25">
+      <c r="H26" s="32">
         <v>88</v>
       </c>
-      <c r="I26" s="38"/>
+      <c r="I26" s="39"/>
     </row>
     <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
+      <c r="A27" s="36">
         <v>60</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="15">
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G27" s="13">
+      <c r="G27" s="18">
         <f t="shared" si="3"/>
         <v>81</v>
       </c>
-      <c r="H27" s="25">
+      <c r="H27" s="32">
         <v>81</v>
       </c>
-      <c r="I27" s="38"/>
+      <c r="I27" s="39"/>
     </row>
     <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="17">
+      <c r="A28" s="36">
         <v>50</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="15">
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G28" s="13">
+      <c r="G28" s="18">
         <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="H28" s="25">
+      <c r="H28" s="32">
         <v>72</v>
       </c>
-      <c r="I28" s="38"/>
+      <c r="I28" s="39"/>
     </row>
     <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="A29" s="36">
         <v>40</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="15">
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="18">
         <f t="shared" si="3"/>
         <v>62</v>
       </c>
-      <c r="H29" s="25">
+      <c r="H29" s="32">
         <v>62</v>
       </c>
-      <c r="I29" s="38"/>
+      <c r="I29" s="39"/>
     </row>
     <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="17">
+      <c r="A30" s="36">
         <v>30</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="15">
+      <c r="B30" s="21"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="18">
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="H30" s="25">
+      <c r="H30" s="32">
         <v>51</v>
       </c>
-      <c r="I30" s="38"/>
+      <c r="I30" s="39"/>
     </row>
     <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17">
+      <c r="A31" s="36">
         <v>20</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="15">
+      <c r="B31" s="21"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="18">
         <f t="shared" si="3"/>
         <v>37</v>
       </c>
-      <c r="H31" s="25">
+      <c r="H31" s="32">
         <v>37</v>
       </c>
-      <c r="I31" s="38"/>
+      <c r="I31" s="39"/>
     </row>
     <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17">
+      <c r="A32" s="36">
         <v>10</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="15">
+      <c r="B32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="18">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="32">
         <v>22</v>
       </c>
-      <c r="I32" s="38"/>
+      <c r="I32" s="39"/>
     </row>
     <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17">
+      <c r="A33" s="36">
         <v>5</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="15">
+      <c r="B33" s="21"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="18">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="H33" s="26">
+      <c r="H33" s="33">
         <v>13</v>
       </c>
-      <c r="I33" s="38"/>
+      <c r="I33" s="39"/>
     </row>
     <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17">
+      <c r="A34" s="36">
         <v>3</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="15">
+      <c r="B34" s="21"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="18">
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="32">
         <v>9</v>
       </c>
-      <c r="I34" s="38"/>
+      <c r="I34" s="39"/>
     </row>
     <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="4">
+      <c r="A35" s="37">
         <v>1</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="7">
+      <c r="B35" s="24"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G35" s="10">
+      <c r="G35" s="27">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H35" s="27">
+      <c r="H35" s="34">
         <v>3</v>
       </c>
-      <c r="I35" s="38"/>
+      <c r="I35" s="39"/>
     </row>
     <row r="36" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="39">
+      <c r="A36" s="16">
         <v>123</v>
       </c>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="32" t="s">
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="38" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1926,7 +2048,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBF39EA-DCD6-490D-96E4-057DAD2F0CCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBF39EA-DCD6-490D-96E4-057DAD2F0CCB}">
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1936,407 +2058,407 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="38">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="39">
         <v>46098</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="38"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="38"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21">
+      <c r="A4" s="35">
         <v>100</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="17">
         <f>SUM(B4:E4)/4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="18">
         <f>-F4+H4</f>
         <v>100</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="31">
         <v>100</v>
       </c>
-      <c r="I4" s="38"/>
+      <c r="I4" s="39"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17">
+      <c r="A5" s="36">
         <v>95</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15">
+      <c r="B5" s="20"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="17">
         <f t="shared" ref="F5:F19" si="0">SUM(B5:E5)/4</f>
         <v>0</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="18">
         <f t="shared" ref="G5:G19" si="1">-F5+H5</f>
         <v>99</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="31">
         <v>99</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="39"/>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
+      <c r="A6" s="36">
         <v>90</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="13">
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="18">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="32">
         <v>97</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="39"/>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17">
+      <c r="A7" s="36">
         <v>80</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="32">
         <v>93</v>
       </c>
-      <c r="I7" s="38"/>
-      <c r="K7" s="22"/>
+      <c r="I7" s="39"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17">
+      <c r="A8" s="36">
         <v>70</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="32">
         <v>88</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="39"/>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
+      <c r="A9" s="36">
         <v>60</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="B9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="32">
         <v>81</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="36">
         <v>50</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="B10" s="21"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="32">
         <v>72</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17">
+      <c r="A11" s="36">
         <v>40</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
+      <c r="B11" s="21"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="32">
         <v>62</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="39"/>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
+      <c r="A12" s="36">
         <v>30</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="32">
         <v>51</v>
       </c>
-      <c r="I12" s="38"/>
+      <c r="I12" s="39"/>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17">
+      <c r="A13" s="36">
         <v>20</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="32">
         <v>37</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="39"/>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+      <c r="A14" s="36">
         <v>10</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="13">
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="32">
         <v>22</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+      <c r="A15" s="36">
         <v>5</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="H15" s="26">
+      <c r="H15" s="33">
         <v>13</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="36">
         <v>3</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="32">
         <v>9</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
+      <c r="A17" s="36">
         <v>1.2</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="13">
+      <c r="B17" s="20"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="H17" s="35">
+      <c r="H17" s="41">
         <v>3</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
+      <c r="A18" s="36">
         <v>0.8</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="13">
+      <c r="B18" s="21"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="H18" s="26">
+      <c r="H18" s="33">
         <v>2</v>
       </c>
-      <c r="I18" s="38"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4">
+      <c r="A19" s="37">
         <v>0.04</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="10">
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="27">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="34">
         <v>1</v>
       </c>
-      <c r="I19" s="38"/>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="39">
+      <c r="A20" s="16">
         <v>123</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="32" t="s">
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="38" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2348,11 +2470,12 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D512DE6C-EB81-44CA-A74B-97F4BB9314F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D512DE6C-EB81-44CA-A74B-97F4BB9314F1}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2365,807 +2488,811 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="38">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="39">
         <v>46098</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="38"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="38"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21">
+      <c r="A4" s="35">
         <v>100</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="17">
         <f>SUM(B4:E4)/4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="18">
         <f>-F4+H4</f>
         <v>100</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="31">
         <v>100</v>
       </c>
-      <c r="I4" s="38"/>
+      <c r="I4" s="39"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17">
+      <c r="A5" s="36">
         <v>95</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15">
+      <c r="B5" s="20"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="17">
         <f t="shared" ref="F5:F19" si="0">SUM(B5:E5)/4</f>
         <v>0</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="18">
         <f t="shared" ref="G5:G19" si="1">-F5+H5</f>
         <v>99</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="31">
         <v>99</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="39"/>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17">
+      <c r="A6" s="36">
         <v>90</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="13">
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="18">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="32">
         <v>97</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="39"/>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17">
+      <c r="A7" s="36">
         <v>80</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="18">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="32">
         <v>93</v>
       </c>
-      <c r="I7" s="38"/>
-      <c r="K7" s="22"/>
+      <c r="I7" s="39"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17">
+      <c r="A8" s="36">
         <v>70</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="13">
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="18">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="32">
         <v>88</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="39"/>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17">
+      <c r="A9" s="36">
         <v>60</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="B9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="32">
         <v>81</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17">
+      <c r="A10" s="36">
         <v>50</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="B10" s="21"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="32">
         <v>72</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17">
+      <c r="A11" s="36">
         <v>40</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
+      <c r="B11" s="21"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="32">
         <v>62</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="39"/>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
+      <c r="A12" s="36">
         <v>30</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="32">
         <v>51</v>
       </c>
-      <c r="I12" s="38"/>
+      <c r="I12" s="39"/>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17">
+      <c r="A13" s="36">
         <v>20</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="32">
         <v>37</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="39"/>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+      <c r="A14" s="36">
         <v>10</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="13">
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="32">
         <v>22</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+      <c r="A15" s="36">
         <v>5</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="H15" s="26">
+      <c r="H15" s="33">
         <v>13</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="36">
         <v>3</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="32">
         <v>9</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
+      <c r="A17" s="36">
         <v>1.2</v>
       </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="13">
+      <c r="B17" s="20"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="41">
         <v>3</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
+      <c r="A18" s="36">
         <v>0.8</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="13">
+      <c r="B18" s="21"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="33">
         <v>2</v>
       </c>
-      <c r="I18" s="38"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="10">
+      <c r="A19" s="37">
+        <v>0.04</v>
+      </c>
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="20">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="27">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="34">
         <v>1</v>
       </c>
-      <c r="I19" s="38"/>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="39">
+      <c r="A20" s="16">
         <v>123</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="32" t="s">
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="38" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="38"/>
+      <c r="A21" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="39">
+        <v>46098</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="28" t="s">
+      <c r="A22" s="2"/>
+      <c r="B22" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="29" t="s">
+      <c r="D22" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E22" s="30" t="s">
+      <c r="E22" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="14" t="s">
+      <c r="G22" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="38"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="21">
+      <c r="A24" s="35">
         <v>100</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="15">
+      <c r="B24" s="17"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="17">
         <f>SUM(B24:E24)/4</f>
         <v>0</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="18">
         <f>-F24+H24</f>
         <v>100</v>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="31">
         <v>100</v>
       </c>
-      <c r="I24" s="38"/>
+      <c r="I24" s="39"/>
     </row>
     <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="17">
+      <c r="A25" s="36">
         <v>95</v>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="15">
+      <c r="B25" s="20"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="17">
         <f t="shared" ref="F25:F39" si="2">SUM(B25:E25)/4</f>
         <v>0</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="18">
         <f t="shared" ref="G25:G39" si="3">-F25+H25</f>
         <v>99</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="31">
         <v>99</v>
       </c>
-      <c r="I25" s="38"/>
+      <c r="I25" s="39"/>
     </row>
     <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
+      <c r="A26" s="36">
         <v>90</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="15">
+      <c r="B26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="18">
         <f t="shared" si="3"/>
         <v>97</v>
       </c>
-      <c r="H26" s="25">
+      <c r="H26" s="32">
         <v>97</v>
       </c>
-      <c r="I26" s="38"/>
+      <c r="I26" s="39"/>
     </row>
     <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
+      <c r="A27" s="36">
         <v>80</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="15">
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G27" s="13">
+      <c r="G27" s="18">
         <f t="shared" si="3"/>
         <v>93</v>
       </c>
-      <c r="H27" s="25">
+      <c r="H27" s="32">
         <v>93</v>
       </c>
-      <c r="I27" s="38"/>
+      <c r="I27" s="39"/>
     </row>
     <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="17">
+      <c r="A28" s="36">
         <v>70</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="15">
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G28" s="13">
+      <c r="G28" s="18">
         <f t="shared" si="3"/>
         <v>88</v>
       </c>
-      <c r="H28" s="25">
+      <c r="H28" s="32">
         <v>88</v>
       </c>
-      <c r="I28" s="38"/>
+      <c r="I28" s="39"/>
     </row>
     <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="A29" s="36">
         <v>60</v>
       </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="15">
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="18">
         <f t="shared" si="3"/>
         <v>81</v>
       </c>
-      <c r="H29" s="25">
+      <c r="H29" s="32">
         <v>81</v>
       </c>
-      <c r="I29" s="38"/>
+      <c r="I29" s="39"/>
     </row>
     <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="17">
+      <c r="A30" s="36">
         <v>50</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="15">
+      <c r="B30" s="21"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G30" s="13">
+      <c r="G30" s="18">
         <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="H30" s="25">
+      <c r="H30" s="32">
         <v>72</v>
       </c>
-      <c r="I30" s="38"/>
+      <c r="I30" s="39"/>
     </row>
     <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17">
+      <c r="A31" s="36">
         <v>40</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="15">
+      <c r="B31" s="21"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G31" s="13">
+      <c r="G31" s="18">
         <f t="shared" si="3"/>
         <v>62</v>
       </c>
-      <c r="H31" s="25">
+      <c r="H31" s="32">
         <v>62</v>
       </c>
-      <c r="I31" s="38"/>
+      <c r="I31" s="39"/>
     </row>
     <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17">
+      <c r="A32" s="36">
         <v>30</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="15">
+      <c r="B32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G32" s="13">
+      <c r="G32" s="18">
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="32">
         <v>51</v>
       </c>
-      <c r="I32" s="38"/>
+      <c r="I32" s="39"/>
     </row>
     <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17">
+      <c r="A33" s="36">
         <v>20</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="15">
+      <c r="B33" s="21"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="18">
         <f t="shared" si="3"/>
         <v>37</v>
       </c>
-      <c r="H33" s="25">
+      <c r="H33" s="32">
         <v>37</v>
       </c>
-      <c r="I33" s="38"/>
+      <c r="I33" s="39"/>
     </row>
     <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17">
+      <c r="A34" s="36">
         <v>10</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="15">
+      <c r="B34" s="21"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G34" s="18">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="32">
         <v>22</v>
       </c>
-      <c r="I34" s="38"/>
+      <c r="I34" s="39"/>
     </row>
     <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17">
+      <c r="A35" s="36">
         <v>5</v>
       </c>
-      <c r="B35" s="18"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="15">
+      <c r="B35" s="21"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G35" s="13">
-        <f>-F35+H35</f>
+      <c r="G35" s="18">
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="H35" s="26">
+      <c r="H35" s="33">
         <v>13</v>
       </c>
-      <c r="I35" s="38"/>
+      <c r="I35" s="39"/>
     </row>
     <row r="36" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="17">
+      <c r="A36" s="36">
         <v>3</v>
       </c>
-      <c r="B36" s="18"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="15">
+      <c r="B36" s="21"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G36" s="13">
-        <f t="shared" ref="G36:G37" si="4">-F36+H36</f>
+      <c r="G36" s="18">
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="H36" s="25">
+      <c r="H36" s="32">
         <v>9</v>
       </c>
-      <c r="I36" s="38"/>
+      <c r="I36" s="39"/>
     </row>
     <row r="37" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17">
+      <c r="A37" s="36">
         <v>1.2</v>
       </c>
-      <c r="B37" s="18"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="15">
+      <c r="B37" s="20"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G37" s="13">
-        <f t="shared" si="4"/>
+      <c r="G37" s="18">
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H37" s="25">
+      <c r="H37" s="41">
         <v>3</v>
       </c>
-      <c r="I37" s="38"/>
+      <c r="I37" s="39"/>
     </row>
     <row r="38" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="17">
+      <c r="A38" s="36">
         <v>0.8</v>
       </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="15">
+      <c r="B38" s="21"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G38" s="13">
+      <c r="G38" s="18">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="H38" s="25">
+      <c r="H38" s="33">
         <v>2</v>
       </c>
-      <c r="I38" s="38"/>
+      <c r="I38" s="39"/>
     </row>
     <row r="39" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="7">
+      <c r="A39" s="37">
+        <v>0.04</v>
+      </c>
+      <c r="B39" s="24"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="20">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G39" s="10">
+      <c r="G39" s="27">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H39" s="27">
+      <c r="H39" s="34">
         <v>1</v>
       </c>
-      <c r="I39" s="38"/>
+      <c r="I39" s="39"/>
     </row>
     <row r="40" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="39">
+      <c r="A40" s="16">
         <v>123</v>
       </c>
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="39"/>
-      <c r="G40" s="39"/>
-      <c r="H40" s="39"/>
-      <c r="I40" s="32" t="s">
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="38" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3180,5 +3307,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="83" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>